<commit_message>
Reset charts.ipynb to match remote repository
</commit_message>
<xml_diff>
--- a/1740CAF(withSheet1).xlsx
+++ b/1740CAF(withSheet1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nehakotha/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nehakotha/GASP-Clean-Air-Fund/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56B515D0-BBDD-C345-A1BD-8619D027820D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3067F339-A806-4043-AA61-6A40F8A9CFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5440" yWindow="760" windowWidth="23360" windowHeight="16300" activeTab="3" xr2:uid="{C5E92D08-1D1E-B946-9078-11755ACCCC10}"/>
   </bookViews>
@@ -11128,7 +11128,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="128">
         <v>2024</v>
       </c>

</xml_diff>